<commit_message>
update lmm with scaling
</commit_message>
<xml_diff>
--- a/results/tab/trait_trait_PS_mixed_model_outputs_raw.xlsx
+++ b/results/tab/trait_trait_PS_mixed_model_outputs_raw.xlsx
@@ -351,954 +351,783 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>part</t>
+          <t>term</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>term</t>
+          <t>statistic</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>statistic</t>
+          <t>A. aboveground biomass~belowground biomass (linear)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>sla~aboveground_biomass_exp</t>
+          <t>B. veg height~root depth (linear)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>srl~aboveground_biomass_exp</t>
+          <t>C. root depth~belowground biomass (linear)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>veg_height~aboveground_biomass_exp</t>
+          <t>D. srl~belowground biomass (linear)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>aboveground_biomass~belowground_biomass_exp</t>
+          <t>E. sla~belowground biomass (polynomial)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>root_depth~belowground_biomass_exp</t>
+          <t>F. veg height~aboveground biomass (polynomial)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>sla~belowground_biomass_exp</t>
+          <t>G. srl~aboveground biomass (linear)</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>srl~belowground_biomass_exp</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>veg_height~root_depth_exp</t>
+          <t>H. sla~aboveground biomass (polynomial)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>estimates</t>
+          <t>Intercept</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>(Intercept)</t>
+          <t>estimate</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>estimate</t>
+          <t>0.055 [0.007, 0.103] *</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>4.901 [4.615, 5.187] ***</t>
+          <t>0.400 [0.226, 0.573] ***</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.317 [4.205, 4.430] ***</t>
+          <t>0.298 [0.226, 0.371] ***</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2.289 [1.802, 2.775] ***</t>
+          <t>0.300 [0.252, 0.348] ***</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0.095 [-0.429, 0.619]</t>
+          <t>0.398 [0.131, 0.664] **</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2.563 [2.432, 2.693] ***</t>
+          <t>0.252 [0.108, 0.397] ***</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>4.923 [4.626, 5.220] ***</t>
+          <t>0.329 [0.285, 0.373] ***</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>4.230 [4.102, 4.358] ***</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2.742 [2.243, 3.241] ***</t>
+          <t>0.375 [0.135, 0.616] **</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>estimates</t>
+          <t>Intercept</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>(Intercept)</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>std.error</t>
+          <t>(0.024)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>(0.144)</t>
+          <t>(0.087)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>(0.057)</t>
+          <t>(0.036)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>(0.245)</t>
+          <t>(0.024)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>(0.264)</t>
+          <t>(0.134)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>(0.066)</t>
+          <t>(0.073)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>(0.149)</t>
+          <t>(0.022)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>(0.064)</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>(0.251)</t>
+          <t>(0.121)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>estimates</t>
+          <t>trait_x</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>aboveground_biomass</t>
+          <t>estimate</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>estimate</t>
+          <t>0.380 [0.170, 0.590] ***</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.014 [0.001, 0.028] *</t>
+          <t>-0.167 [-0.371, 0.038]</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>-0.035 [-0.062, -0.008] *</t>
+          <t>0.223 [-0.007, 0.453] +</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.059 [-0.031, 0.148]</t>
+          <t>-0.024 [-0.188, 0.139]</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>-0.358 [-0.840, 0.124]</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0.906 [0.353, 1.460] **</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>-0.241 [-0.437, -0.045] *</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>-0.266 [-0.751, 0.218]</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>estimates</t>
+          <t>trait_x</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>aboveground_biomass</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>std.error</t>
+          <t>(0.105)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>(0.007)</t>
+          <t>(0.103)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>(0.014)</t>
+          <t>(0.116)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>(0.045)</t>
+          <t>(0.082)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(0.242)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>(0.278)</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>(0.099)</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>(0.244)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>estimates</t>
+          <t>I(trait_x^2)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>belowground_biomass</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
           <t>estimate</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0.081 [0.045, 0.117] ***</t>
+          <t>0.687 [0.168, 1.206] *</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>0.010 [0.001, 0.019] *</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>0.004 [-0.003, 0.010]</t>
+          <t>-0.978 [-1.595, -0.360] **</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>-0.002 [-0.016, 0.011]</t>
+          <t>0.607 [0.036, 1.177] *</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>estimates</t>
+          <t>I(trait_x^2)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>belowground_biomass</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>std.error</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>(0.018)</t>
+          <t>(0.261)</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>(0.005)</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>(0.003)</t>
+          <t>(0.311)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>(0.007)</t>
+          <t>(0.287)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>estimates</t>
+          <t>SD (Intercept species)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>root_depth</t>
+          <t>estimate</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>estimate</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>-0.023 [-0.042, -0.004] *</t>
+          <t>0.029</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0.180</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0.057</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.293</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0.152</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>0.265</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>estimates</t>
+          <t>SD (trait_x species)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>root_depth</t>
+          <t>estimate</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>std.error</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>(0.010)</t>
+          <t>0.125</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0.129</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0.102</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0.238</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>0.331</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>0.109</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>estimates</t>
+          <t>Cor (Intercept~trait_x species)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SD (Intercept species)</t>
+          <t>estimate</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>estimate</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.318</t>
+          <t>-1.000</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0.538</t>
+          <t>-0.904</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0.548</t>
+          <t>-1.000</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>0.115</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>0.330</t>
+          <t>-1.000</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>0.039</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>0.461</t>
+          <t>-1.000</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>estimates</t>
+          <t>SD (Observations)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>SD (aboveground_biomass species)</t>
+          <t>estimate</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>estimate</t>
+          <t>0.128</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.008</t>
+          <t>0.138</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.165</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0.096</t>
+          <t>0.168</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>0.126</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>0.130</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>0.163</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>0.126</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>estimates</t>
+          <t>Num.Obs.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Cor (Intercept~aboveground_biomass species)</t>
+          <t>statistic</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>estimate</t>
+          <t>91</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-1.000</t>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>91</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-0.990</t>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>91</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>estimates</t>
+          <t>R2 Marg.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SD (belowground_biomass species)</t>
+          <t>statistic</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>estimate</t>
+          <t>0.289</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>0.054</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>0.078</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>0.001</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>0.032</t>
+          <t>0.142</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>0.002</t>
+          <t>0.187</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>0.004</t>
+          <t>0.062</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>0.005</t>
+          <t>0.099</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>estimates</t>
+          <t>AIC</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cor (Intercept~belowground_biomass species)</t>
+          <t>statistic</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>estimate</t>
+          <t>-88.0</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>-68.3</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>-42.5</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>-45.3</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-0.928</t>
+          <t>-75.9</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>-77.1</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>-1.000</t>
+          <t>-51.3</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>-1.000</t>
+          <t>-77.8</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>estimates</t>
+          <t>BIC</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SD (root_depth species)</t>
+          <t>statistic</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>estimate</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>0.003</t>
+          <t>-73.0</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>-53.2</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>-27.4</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>-30.2</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>-58.3</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>-59.6</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>-36.2</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>-60.2</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>estimates</t>
+          <t>RMSE</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Cor (Intercept~root_depth species)</t>
+          <t>statistic</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>estimate</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>-1.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>estimates</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>SD (Observations)</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>estimate</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>0.148</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>0.402</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>0.300</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>0.592</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>0.254</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>0.151</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>0.415</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>0.334</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>gof</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Num.Obs.</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>91</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>91</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>91</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>91</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>91</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>91</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>91</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>91</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>gof</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>R2 Marg.</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>0.084</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>0.071</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>0.117</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>0.398</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>0.072</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>0.029</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>0.002</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>0.082</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>gof</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>R2 Cond.</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>0.687</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>0.597</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>gof</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>AIC</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>758.2</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>975.3</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>550.0</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>461.7</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>526.8</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>767.2</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>988.4</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>588.4</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>gof</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>BIC</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>773.3</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>990.4</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>565.1</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>476.8</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>541.9</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>782.2</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>1003.4</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>603.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>gof</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>ICC</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>0.6</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>0.3</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>gof</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>RMSE</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>0.14</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>0.40</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>0.29</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>0.57</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>0.25</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>0.15</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>0.41</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>0.32</t>
+          <t>0.13</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>0.13</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0.16</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0.17</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>0.12</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>0.13</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>0.16</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>0.12</t>
         </is>
       </c>
     </row>

</xml_diff>